<commit_message>
Final corrections to First order logic notes
</commit_message>
<xml_diff>
--- a/kb-book/Part1/Einstein Puzzle.xlsx
+++ b/kb-book/Part1/Einstein Puzzle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qubstudentcloud-my.sharepoint.com/personal/3057867_ads_qub_ac_uk/Documents/GIT/Knowledge-Engineering-2025/kb-book/Part1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FA86F33-6484-A04E-8368-FEE8C176C14F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="446" documentId="8_{2FA86F33-6484-A04E-8368-FEE8C176C14F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90D4FA89-823E-8B4B-9C8D-4E22201E81D9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{B12FA4F3-C76C-8D41-8190-B337A8B4EE53}"/>
+    <workbookView xWindow="1020" yWindow="740" windowWidth="28380" windowHeight="18380" xr2:uid="{B12FA4F3-C76C-8D41-8190-B337A8B4EE53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="45">
   <si>
     <t>Milk</t>
   </si>
@@ -162,6 +162,15 @@
   </si>
   <si>
     <t>The Norwegian lives next to the blue house.</t>
+  </si>
+  <si>
+    <t>Chest</t>
+  </si>
+  <si>
+    <t>Lucky</t>
+  </si>
+  <si>
+    <t>Parl</t>
   </si>
 </sst>
 </file>
@@ -195,18 +204,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="9">
@@ -301,31 +304,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,7 +684,7 @@
   <dimension ref="A1:AD27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="104" style="11" customWidth="1"/>
+    <col min="1" max="1" width="92.1640625" style="9" customWidth="1"/>
     <col min="6" max="7" width="5.5" customWidth="1"/>
     <col min="8" max="8" width="4.5" customWidth="1"/>
     <col min="9" max="9" width="4" customWidth="1"/>
@@ -709,12 +709,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F2" t="s">
@@ -794,7 +794,7 @@
       </c>
     </row>
     <row r="3" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>35</v>
       </c>
       <c r="E3">
@@ -815,35 +815,69 @@
       <c r="J3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="1"/>
+      <c r="K3" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="L3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="2"/>
+      <c r="M3" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="N3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="3"/>
+      <c r="O3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="Z3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
-      <c r="AC3" s="2"/>
-      <c r="AD3" s="3"/>
+      <c r="AA3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD3" s="3" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>36</v>
       </c>
       <c r="E4">
@@ -852,51 +886,81 @@
       <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="5"/>
-      <c r="J4" s="6"/>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="K4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="6"/>
+      <c r="L4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="S4" t="s">
+        <v>25</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="U4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="6"/>
-      <c r="Z4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="5"/>
-      <c r="AC4" s="5"/>
-      <c r="AD4" s="6" t="s">
+      <c r="V4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD4" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="11" t="s">
         <v>27</v>
       </c>
       <c r="E5">
@@ -905,40 +969,76 @@
       <c r="F5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O5" s="6"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="6"/>
-      <c r="Z5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC5" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="AD5" s="6" t="s">
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" t="s">
+        <v>26</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="S5" t="s">
+        <v>26</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="W5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="X5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z5" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD5" s="5" t="s">
         <v>26</v>
       </c>
     </row>
@@ -952,78 +1052,164 @@
       <c r="F6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" s="6"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="6"/>
-      <c r="Z6" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA6" s="5"/>
-      <c r="AB6" s="5"/>
-      <c r="AC6" s="5"/>
-      <c r="AD6" s="6"/>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" t="s">
+        <v>26</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="S6" t="s">
+        <v>26</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="V6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="W6" t="s">
+        <v>25</v>
+      </c>
+      <c r="X6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC6" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="AD6" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="7" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="11" t="s">
         <v>28</v>
       </c>
       <c r="E7">
         <v>5</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="O7" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="7"/>
-      <c r="V7" s="8"/>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8"/>
-      <c r="Y7" s="9"/>
-      <c r="Z7" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA7" s="8"/>
-      <c r="AB7" s="8"/>
-      <c r="AC7" s="8"/>
-      <c r="AD7" s="9"/>
+      <c r="F7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="T7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD7" s="8" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="12" t="s">
         <v>38</v>
       </c>
       <c r="E8" t="s">
@@ -1032,70 +1218,134 @@
       <c r="F8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="G8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="J8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="L8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M8" s="2"/>
+      <c r="M8" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="N8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="2"/>
+      <c r="O8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="W8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="3"/>
+      <c r="X8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="11" t="s">
         <v>29</v>
       </c>
       <c r="E9" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K9" s="4"/>
-      <c r="L9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="4"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="X9" s="5"/>
-      <c r="Y9" s="6"/>
+      <c r="F9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="S9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="T9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="V9" t="s">
+        <v>26</v>
+      </c>
+      <c r="W9" t="s">
+        <v>26</v>
+      </c>
+      <c r="X9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="10" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="12" t="s">
         <v>39</v>
       </c>
       <c r="E10" t="s">
@@ -1104,146 +1354,222 @@
       <c r="F10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J10" s="6" t="s">
+      <c r="G10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="5" t="s">
         <v>25</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M10" s="10"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="5"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="4"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="X10" s="5"/>
-      <c r="Y10" s="6"/>
+      <c r="L10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S10" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="T10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="V10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="W10" t="s">
+        <v>26</v>
+      </c>
+      <c r="X10" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="11" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="11" t="s">
         <v>30</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="6"/>
+      <c r="F11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R11" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="S11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="T11" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="U11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="V11" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="W11" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="X11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y11" s="6" t="s">
+      <c r="V11" t="s">
+        <v>26</v>
+      </c>
+      <c r="W11" t="s">
+        <v>25</v>
+      </c>
+      <c r="X11" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y11" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="11" t="s">
         <v>31</v>
       </c>
       <c r="E12" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="N12" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="O12" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="9"/>
+      <c r="F12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="S12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="T12" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="V12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="W12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="X12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y12" s="8" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="13" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>40</v>
       </c>
       <c r="E13" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
+      <c r="F13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="H13" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J13" s="3"/>
+      <c r="J13" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="K13" s="1" t="s">
         <v>26</v>
       </c>
@@ -1262,47 +1588,69 @@
       <c r="P13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
+      <c r="Q13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="S13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="T13" s="3"/>
+      <c r="T13" s="3" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="14" spans="1:30" ht="23" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="11" t="s">
         <v>32</v>
       </c>
       <c r="E14" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N14" s="5"/>
-      <c r="O14" s="6"/>
+      <c r="F14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" t="s">
+        <v>26</v>
+      </c>
+      <c r="N14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O14" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="P14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="R14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="S14" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="T14" s="6" t="s">
+      <c r="Q14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R14" t="s">
+        <v>26</v>
+      </c>
+      <c r="S14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="T14" s="5" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1313,192 +1661,425 @@
       <c r="E15" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K15" s="4"/>
-      <c r="L15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N15" s="5"/>
-      <c r="O15" s="6"/>
+      <c r="F15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" t="s">
+        <v>26</v>
+      </c>
+      <c r="N15" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="P15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="6"/>
+      <c r="Q15" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R15" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="S15" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="T15" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A16" s="13"/>
       <c r="E16" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N16" s="5"/>
-      <c r="O16" s="6"/>
+      <c r="G16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H16" t="s">
+        <v>26</v>
+      </c>
+      <c r="I16" t="s">
+        <v>25</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" t="s">
+        <v>26</v>
+      </c>
+      <c r="N16" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="P16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="5"/>
-      <c r="S16" s="5"/>
-      <c r="T16" s="6"/>
-    </row>
-    <row r="17" spans="5:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="Q16" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R16" t="s">
+        <v>26</v>
+      </c>
+      <c r="S16" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="T16" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13"/>
       <c r="E17" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="7"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="J17" s="9"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="N17" s="8"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q17" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="9"/>
-    </row>
-    <row r="18" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="F17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O17" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="T17" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="W17">
+        <v>1</v>
+      </c>
+      <c r="X17" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A18" s="13"/>
       <c r="E18" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="G18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="I18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J18" s="3"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="3"/>
-    </row>
-    <row r="19" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="J18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="W18">
+        <v>2</v>
+      </c>
+      <c r="X18" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>7</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A19" s="13"/>
       <c r="E19" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="6"/>
-    </row>
-    <row r="20" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="F19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="N19" t="s">
+        <v>26</v>
+      </c>
+      <c r="O19" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="W19">
+        <v>3</v>
+      </c>
+      <c r="X19" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>2</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A20" s="13"/>
       <c r="E20" t="s">
         <v>5</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J20" s="6" t="s">
+      <c r="G20" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J20" s="5" t="s">
         <v>26</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="L20" s="5"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="6"/>
-    </row>
-    <row r="21" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="L20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="N20" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="W20">
+        <v>4</v>
+      </c>
+      <c r="X20" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A21" s="13"/>
       <c r="E21" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="6"/>
-    </row>
-    <row r="22" spans="5:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L21" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+      <c r="O21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="W21">
+        <v>5</v>
+      </c>
+      <c r="X21" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13"/>
       <c r="E22" t="s">
         <v>8</v>
       </c>
-      <c r="F22" s="7"/>
-      <c r="G22" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="9"/>
-    </row>
-    <row r="23" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
       <c r="E23" t="s">
         <v>2</v>
       </c>
@@ -1518,61 +2099,85 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="5:20" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
       <c r="E24" t="s">
         <v>3</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I24" s="5"/>
-      <c r="J24" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="G24" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H24" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
       <c r="E25" t="s">
         <v>4</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J25" s="6"/>
-    </row>
-    <row r="26" spans="5:20" x14ac:dyDescent="0.2">
+      <c r="F25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
       <c r="E26" t="s">
         <v>1</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G26" s="5"/>
-      <c r="H26" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="6"/>
-    </row>
-    <row r="27" spans="5:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" t="s">
+        <v>26</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E27" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="7"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I27" s="8"/>
-      <c r="J27" s="9"/>
+      <c r="F27" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F3:AD27">

</xml_diff>